<commit_message>
feat(evaluator): harden enterprise physical aspects, universal knowledge charter, and CLIC validation invariants (INV-25 to INV-29)
</commit_message>
<xml_diff>
--- a/outputs/ProLiant/Gen11/DL380_Gen11/HPE_DL380_Gen11_PartnerPortal_BOM_GID-RFQS-HPE-2026-006.xlsx
+++ b/outputs/ProLiant/Gen11/DL380_Gen11/HPE_DL380_Gen11_PartnerPortal_BOM_GID-RFQS-HPE-2026-006.xlsx
@@ -752,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F61"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -931,27 +931,27 @@
         <v>Thermal</v>
       </c>
       <c r="C9" s="13" t="str">
-        <v>HPE ProLiant DL380/DL560 Gen11 2U High Performance Fan Kit</v>
+        <v>HPE ProLiant DL380/DL560 Gen11 2U High Performance Fan Kit (All 6 Fans)</v>
       </c>
       <c r="D9" s="14">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E9" s="11" t="str">
         <v/>
       </c>
       <c r="F9" s="14">
-        <v>120</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="str">
-        <v>P64707-B21</v>
+        <v>P64707-B21 0D1</v>
       </c>
       <c r="B10" s="9" t="str">
         <v>Memory</v>
       </c>
       <c r="C10" s="9" t="str">
-        <v>HPE 64GB (1x64GB) Dual Rank x4 DDR5-5600 CAS-46-45-45 EC8 Registered Smart Memory Kit</v>
+        <v>HPE 64GB (1x64GB) Dual Rank x4 DDR5-5600 CAS-46-45-45 EC8 Registered Smart FIO Memory Kit</v>
       </c>
       <c r="D10" s="10">
         <v>8</v>
@@ -1008,7 +1008,7 @@
         <v>P02377-B21</v>
       </c>
       <c r="B13" s="13" t="str">
-        <v>Storage Controller</v>
+        <v>Storage Battery</v>
       </c>
       <c r="C13" s="13" t="str">
         <v>HPE Smart Storage Hybrid Capacitor with 145mm Cable Kit</v>
@@ -1025,13 +1025,13 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="str">
-        <v>P48183-B21</v>
+        <v>P48918-B21</v>
       </c>
       <c r="B14" s="9" t="str">
-        <v>Boot Device</v>
+        <v>Storage Cable</v>
       </c>
       <c r="C14" s="9" t="str">
-        <v>HPE NS204i-u Gen11 NVMe Hot Plug Boot Optimized Storage Device</v>
+        <v>HPE ProLiant DL380 Gen11 Storage Controller Enablement Cable Kit (for MR408i-o)</v>
       </c>
       <c r="D14" s="10">
         <v>1</v>
@@ -1045,13 +1045,13 @@
     </row>
     <row r="15">
       <c r="A15" s="12" t="str">
-        <v>P52152-B21</v>
+        <v>P48183-B21</v>
       </c>
       <c r="B15" s="13" t="str">
         <v>Boot Device</v>
       </c>
       <c r="C15" s="13" t="str">
-        <v>HPE ProLiant DL380 Gen11 NS204i-u Internal 40 Cable Kit</v>
+        <v>HPE NS204i-u Gen11 NVMe Hot Plug Boot Optimized Storage Device</v>
       </c>
       <c r="D15" s="14">
         <v>1</v>
@@ -1065,13 +1065,13 @@
     </row>
     <row r="16">
       <c r="A16" s="8" t="str">
-        <v>P54542-B21</v>
+        <v>P52152-B21</v>
       </c>
       <c r="B16" s="9" t="str">
         <v>Boot Device</v>
       </c>
       <c r="C16" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 NS204i-u FIO Bundle Kit</v>
+        <v>HPE ProLiant DL380 Gen11 NS204i-u Internal 40 Cable Kit</v>
       </c>
       <c r="D16" s="10">
         <v>1</v>
@@ -1085,13 +1085,13 @@
     </row>
     <row r="17">
       <c r="A17" s="12" t="str">
-        <v>P48813-B21</v>
+        <v>P54542-B21</v>
       </c>
       <c r="B17" s="13" t="str">
-        <v>Drive Cage</v>
+        <v>Boot Device</v>
       </c>
       <c r="C17" s="13" t="str">
-        <v>HPE ProLiant DL380 Gen11 2U 8SFF x1 Tri-Mode U.3 Drive Cage Kit</v>
+        <v>HPE ProLiant DL380 Gen11 NS204i-u FIO Bundle Kit</v>
       </c>
       <c r="D17" s="14">
         <v>1</v>
@@ -1105,13 +1105,13 @@
     </row>
     <row r="18">
       <c r="A18" s="8" t="str">
-        <v>P48832-B21</v>
+        <v>P48813-B21</v>
       </c>
       <c r="B18" s="9" t="str">
-        <v>Storage Cable</v>
+        <v>Drive Cage</v>
       </c>
       <c r="C18" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 Tri-Mode Splitter Cable Kit</v>
+        <v>HPE ProLiant DL380 Gen11 2U 8SFF x1 Tri-Mode U.3 Drive Cage Kit</v>
       </c>
       <c r="D18" s="10">
         <v>1</v>
@@ -1125,13 +1125,13 @@
     </row>
     <row r="19">
       <c r="A19" s="12" t="str">
-        <v>P51911-B21</v>
+        <v>P48830-B21</v>
       </c>
       <c r="B19" s="13" t="str">
         <v>OCP Enablement</v>
       </c>
       <c r="C19" s="13" t="str">
-        <v>HPE ProLiant DL360 Gen11 CPU1 to OCP2 x8 Enablement Kit</v>
+        <v>HPE ProLiant DL3XX Gen11 CPU2 to OCP2 x8 Enablement Kit</v>
       </c>
       <c r="D19" s="14">
         <v>1</v>
@@ -1145,13 +1145,13 @@
     </row>
     <row r="20">
       <c r="A20" s="8" t="str">
-        <v>P48830-B21</v>
+        <v>P51181-B21</v>
       </c>
       <c r="B20" s="9" t="str">
-        <v>OCP Enablement</v>
+        <v>Network Adapter</v>
       </c>
       <c r="C20" s="9" t="str">
-        <v>HPE ProLiant DL3XX Gen11 CPU2 to OCP2 x8 Enablement Kit</v>
+        <v>Broadcom BCM5719 Ethernet 1Gb 4-port BASE-T OCP3 Adapter for HPE</v>
       </c>
       <c r="D20" s="10">
         <v>1</v>
@@ -1165,13 +1165,13 @@
     </row>
     <row r="21">
       <c r="A21" s="12" t="str">
-        <v>P51181-B21</v>
+        <v>P10115-B21</v>
       </c>
       <c r="B21" s="13" t="str">
         <v>Network Adapter</v>
       </c>
       <c r="C21" s="13" t="str">
-        <v>Broadcom BCM5719 Ethernet 1Gb 4-port BASE-T OCP3 Adapter for HPE</v>
+        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 OCP3 Adapter for HPE</v>
       </c>
       <c r="D21" s="14">
         <v>1</v>
@@ -1185,93 +1185,93 @@
     </row>
     <row r="22">
       <c r="A22" s="8" t="str">
-        <v>P10115-B21</v>
+        <v>P26262-B21</v>
       </c>
       <c r="B22" s="9" t="str">
         <v>Network Adapter</v>
       </c>
       <c r="C22" s="9" t="str">
-        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 OCP3 Adapter for HPE</v>
+        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 Adapter for HPE</v>
       </c>
       <c r="D22" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E22" s="11" t="str">
         <v/>
       </c>
       <c r="F22" s="10">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="12" t="str">
-        <v>P26262-B21</v>
+        <v>845398-B21</v>
       </c>
       <c r="B23" s="13" t="str">
-        <v>Network Adapter</v>
+        <v>Transceiver</v>
       </c>
       <c r="C23" s="13" t="str">
-        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 Adapter for HPE</v>
+        <v>HPE 25Gb SFP28 SR 100m Transceiver</v>
       </c>
       <c r="D23" s="14">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E23" s="11" t="str">
         <v/>
       </c>
       <c r="F23" s="14">
-        <v>40</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="str">
-        <v>845398-B21</v>
+        <v>R2E09A</v>
       </c>
       <c r="B24" s="9" t="str">
-        <v>Transceiver</v>
+        <v>FC HBA</v>
       </c>
       <c r="C24" s="9" t="str">
-        <v>HPE 25Gb SFP28 SR 100m Transceiver</v>
+        <v>HPE SN1610Q 32Gb 2-port Fiber Channel Host Bus Adapter</v>
       </c>
       <c r="D24" s="10">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E24" s="11" t="str">
         <v/>
       </c>
       <c r="F24" s="10">
-        <v>120</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="str">
-        <v>R2E09A</v>
+        <v>P48803-B21</v>
       </c>
       <c r="B25" s="13" t="str">
-        <v>FC HBA</v>
+        <v>PCIe Riser</v>
       </c>
       <c r="C25" s="13" t="str">
-        <v>HPE SN1610Q 32Gb 2-port Fiber Channel Host Bus Adapter</v>
+        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Primary Riser Kit</v>
       </c>
       <c r="D25" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="11" t="str">
         <v/>
       </c>
       <c r="F25" s="14">
-        <v>40</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="str">
-        <v>P48803-B21</v>
+        <v>P56073-B21</v>
       </c>
       <c r="B26" s="9" t="str">
-        <v>PCIe Riser</v>
+        <v>PCIe Riser Cable</v>
       </c>
       <c r="C26" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Primary Riser Kit</v>
+        <v>HPE ProLiant DL380 Gen11 x16/x16/x16 Primary Cable Kit (Slot 1 Enablement)</v>
       </c>
       <c r="D26" s="10">
         <v>1</v>
@@ -1305,13 +1305,13 @@
     </row>
     <row r="28">
       <c r="A28" s="8" t="str">
-        <v>P52341-B21</v>
+        <v>P56074-B21</v>
       </c>
       <c r="B28" s="9" t="str">
-        <v>Racking</v>
+        <v>PCIe Riser Cable</v>
       </c>
       <c r="C28" s="9" t="str">
-        <v>HPE ProLiant DL3XX Gen11 Easy Install Rail 3 Kit</v>
+        <v>HPE ProLiant DL380 Gen11 x16/x16/x16 Secondary Cable Kit (Slot 4 Enablement)</v>
       </c>
       <c r="D28" s="10">
         <v>1</v>
@@ -1325,13 +1325,13 @@
     </row>
     <row r="29">
       <c r="A29" s="12" t="str">
-        <v>P22020-B21</v>
+        <v>P52341-B21</v>
       </c>
       <c r="B29" s="13" t="str">
         <v>Racking</v>
       </c>
       <c r="C29" s="13" t="str">
-        <v>HPE DL38X Gen10 Plus 2U Cable Management Arm for Rail Kit</v>
+        <v>HPE ProLiant DL3XX Gen11 Easy Install Rail 3 Kit</v>
       </c>
       <c r="D29" s="14">
         <v>1</v>
@@ -1344,255 +1344,255 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E30" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F30" s="2" t="str">
-        <v/>
+      <c r="A30" s="8" t="str">
+        <v>P22020-B21</v>
+      </c>
+      <c r="B30" s="9" t="str">
+        <v>Racking</v>
+      </c>
+      <c r="C30" s="9" t="str">
+        <v>HPE DL38X Gen10 Plus 2U Cable Management Arm for Rail Kit</v>
+      </c>
+      <c r="D30" s="10">
+        <v>1</v>
+      </c>
+      <c r="E30" s="11" t="str">
+        <v/>
+      </c>
+      <c r="F30" s="10">
+        <v>20</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="B31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="C31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="D31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="E31" s="2" t="str">
-        <v/>
-      </c>
-      <c r="F31" s="2" t="str">
-        <v/>
+      <c r="A31" s="12" t="str">
+        <v>R7A11AAE</v>
+      </c>
+      <c r="B31" s="13" t="str">
+        <v>Management License</v>
+      </c>
+      <c r="C31" s="13" t="str">
+        <v>HPE Compute Ops Management Enhanced 3-year SaaS</v>
+      </c>
+      <c r="D31" s="14">
+        <v>1</v>
+      </c>
+      <c r="E31" s="11" t="str">
+        <v/>
+      </c>
+      <c r="F31" s="14">
+        <v>20</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="str">
+      <c r="A32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E32" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F32" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="B33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="C33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="D33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="E33" s="2" t="str">
+        <v/>
+      </c>
+      <c r="F33" s="2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="str">
         <v>CONFIGURATION 2: Dense Gold Compute Workload Cluster (40x Nodes | Dual Xeon-Gold 6530 32C 270W)</v>
       </c>
-      <c r="B32" s="15" t="str">
-        <v/>
-      </c>
-      <c r="C32" s="15" t="str">
-        <v/>
-      </c>
-      <c r="D32" s="15" t="str">
-        <v/>
-      </c>
-      <c r="E32" s="15" t="str">
-        <v/>
-      </c>
-      <c r="F32" s="15" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="str">
+      <c r="B34" s="15" t="str">
+        <v/>
+      </c>
+      <c r="C34" s="15" t="str">
+        <v/>
+      </c>
+      <c r="D34" s="15" t="str">
+        <v/>
+      </c>
+      <c r="E34" s="15" t="str">
+        <v/>
+      </c>
+      <c r="F34" s="15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="str">
         <v>Part Number (SKU)</v>
       </c>
-      <c r="B33" s="7" t="str">
+      <c r="B35" s="7" t="str">
         <v>Category</v>
       </c>
-      <c r="C33" s="7" t="str">
+      <c r="C35" s="7" t="str">
         <v>Description</v>
       </c>
-      <c r="D33" s="7" t="str">
+      <c r="D35" s="7" t="str">
         <v>Qty (Per Node)</v>
       </c>
-      <c r="E33" s="7" t="str">
+      <c r="E35" s="7" t="str">
         <v>Set / Multiplier</v>
       </c>
-      <c r="F33" s="7" t="str">
+      <c r="F35" s="7" t="str">
         <v>Total Order Qty</v>
       </c>
     </row>
-    <row r="34" xml:space="preserve">
-      <c r="A34" s="8" t="str">
+    <row r="36" xml:space="preserve">
+      <c r="A36" s="8" t="str">
         <v>P52534-B21</v>
       </c>
-      <c r="B34" s="9" t="str">
+      <c r="B36" s="9" t="str">
         <v>Base Chassis</v>
       </c>
-      <c r="C34" s="9" t="str">
+      <c r="C36" s="9" t="str">
         <v>HPE ProLiant DL380 Gen11 8SFF NC Configure-to-order Server</v>
       </c>
-      <c r="D34" s="10">
-        <v>1</v>
-      </c>
-      <c r="E34" s="16" t="str" xml:space="preserve">
+      <c r="D36" s="10">
+        <v>1</v>
+      </c>
+      <c r="E36" s="16" t="str" xml:space="preserve">
         <v xml:space="preserve">40x Server Nodes
 (Multiplier: 40)</v>
       </c>
-      <c r="F34" s="10">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="str">
-        <v>P67095-B21</v>
-      </c>
-      <c r="B35" s="13" t="str">
-        <v>Processor</v>
-      </c>
-      <c r="C35" s="13" t="str">
-        <v>Intel Xeon-Gold 6530 2.1GHz 32-core 270W Processor for HPE</v>
-      </c>
-      <c r="D35" s="14">
-        <v>2</v>
-      </c>
-      <c r="E35" s="16" t="str">
-        <v/>
-      </c>
-      <c r="F35" s="14">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="str">
-        <v>P48818-B21</v>
-      </c>
-      <c r="B36" s="9" t="str">
-        <v>Thermal</v>
-      </c>
-      <c r="C36" s="9" t="str">
-        <v>HPE ProLiant DL380/DL560 Gen11 High-performance 2U Heat Sink Kit</v>
-      </c>
-      <c r="D36" s="10">
-        <v>2</v>
-      </c>
-      <c r="E36" s="16" t="str">
-        <v/>
-      </c>
       <c r="F36" s="10">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="12" t="str">
-        <v>P48820-B21</v>
+        <v>P67095-B21</v>
       </c>
       <c r="B37" s="13" t="str">
-        <v>Thermal</v>
+        <v>Processor</v>
       </c>
       <c r="C37" s="13" t="str">
-        <v>HPE ProLiant DL380/DL560 Gen11 2U High Performance Fan Kit</v>
+        <v>Intel Xeon-Gold 6530 2.1GHz 32-core 270W Processor for HPE</v>
       </c>
       <c r="D37" s="14">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E37" s="16" t="str">
         <v/>
       </c>
       <c r="F37" s="14">
-        <v>240</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="str">
-        <v>P64707-B21</v>
+        <v>P48818-B21</v>
       </c>
       <c r="B38" s="9" t="str">
-        <v>Memory</v>
+        <v>Thermal</v>
       </c>
       <c r="C38" s="9" t="str">
-        <v>HPE 64GB (1x64GB) Dual Rank x4 DDR5-5600 CAS-46-45-45 EC8 Registered Smart Memory Kit</v>
+        <v>HPE ProLiant DL380/DL560 Gen11 High-performance 2U Heat Sink Kit</v>
       </c>
       <c r="D38" s="10">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E38" s="16" t="str">
         <v/>
       </c>
       <c r="F38" s="10">
-        <v>320</v>
+        <v>80</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="str">
-        <v>P38997-B21</v>
+        <v>P48820-B21</v>
       </c>
       <c r="B39" s="13" t="str">
-        <v>Power Supply</v>
+        <v>Thermal</v>
       </c>
       <c r="C39" s="13" t="str">
-        <v>HPE 1600W Flex Slot Platinum Hot Plug Low Halogen Power Supply Kit</v>
+        <v>HPE ProLiant DL380/DL560 Gen11 2U High Performance Fan Kit (All 6 Fans)</v>
       </c>
       <c r="D39" s="14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" s="16" t="str">
         <v/>
       </c>
       <c r="F39" s="14">
-        <v>80</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="str">
-        <v>P58335-B21</v>
+        <v>P64707-B21 0D1</v>
       </c>
       <c r="B40" s="9" t="str">
-        <v>Storage Controller</v>
+        <v>Memory</v>
       </c>
       <c r="C40" s="9" t="str">
-        <v>HPE MR408i-o Gen11 x8 Lanes 4GB Cache OCP SPDM Storage Controller</v>
+        <v>HPE 64GB (1x64GB) Dual Rank x4 DDR5-5600 CAS-46-45-45 EC8 Registered Smart FIO Memory Kit</v>
       </c>
       <c r="D40" s="10">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E40" s="16" t="str">
         <v/>
       </c>
       <c r="F40" s="10">
-        <v>40</v>
+        <v>320</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="12" t="str">
-        <v>P02377-B21</v>
+        <v>P38997-B21</v>
       </c>
       <c r="B41" s="13" t="str">
-        <v>Storage Controller</v>
+        <v>Power Supply</v>
       </c>
       <c r="C41" s="13" t="str">
-        <v>HPE Smart Storage Hybrid Capacitor with 145mm Cable Kit</v>
+        <v>HPE 1600W Flex Slot Platinum Hot Plug Low Halogen Power Supply Kit</v>
       </c>
       <c r="D41" s="14">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E41" s="16" t="str">
         <v/>
       </c>
       <c r="F41" s="14">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="str">
-        <v>P48183-B21</v>
+        <v>P58335-B21</v>
       </c>
       <c r="B42" s="9" t="str">
-        <v>Boot Device</v>
+        <v>Storage Controller</v>
       </c>
       <c r="C42" s="9" t="str">
-        <v>HPE NS204i-u Gen11 NVMe Hot Plug Boot Optimized Storage Device</v>
+        <v>HPE MR408i-o Gen11 x8 Lanes 4GB Cache OCP SPDM Storage Controller</v>
       </c>
       <c r="D42" s="10">
         <v>1</v>
@@ -1606,13 +1606,13 @@
     </row>
     <row r="43">
       <c r="A43" s="12" t="str">
-        <v>P52152-B21</v>
+        <v>P02377-B21</v>
       </c>
       <c r="B43" s="13" t="str">
-        <v>Boot Device</v>
+        <v>Storage Battery</v>
       </c>
       <c r="C43" s="13" t="str">
-        <v>HPE ProLiant DL380 Gen11 NS204i-u Internal 40 Cable Kit</v>
+        <v>HPE Smart Storage Hybrid Capacitor with 145mm Cable Kit</v>
       </c>
       <c r="D43" s="14">
         <v>1</v>
@@ -1626,13 +1626,13 @@
     </row>
     <row r="44">
       <c r="A44" s="8" t="str">
-        <v>P54542-B21</v>
+        <v>P48918-B21</v>
       </c>
       <c r="B44" s="9" t="str">
-        <v>Boot Device</v>
+        <v>Storage Cable</v>
       </c>
       <c r="C44" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 NS204i-u FIO Bundle Kit</v>
+        <v>HPE ProLiant DL380 Gen11 Storage Controller Enablement Cable Kit (for MR408i-o)</v>
       </c>
       <c r="D44" s="10">
         <v>1</v>
@@ -1646,13 +1646,13 @@
     </row>
     <row r="45">
       <c r="A45" s="12" t="str">
-        <v>P48813-B21</v>
+        <v>P48183-B21</v>
       </c>
       <c r="B45" s="13" t="str">
-        <v>Drive Cage</v>
+        <v>Boot Device</v>
       </c>
       <c r="C45" s="13" t="str">
-        <v>HPE ProLiant DL380 Gen11 2U 8SFF x1 Tri-Mode U.3 Drive Cage Kit</v>
+        <v>HPE NS204i-u Gen11 NVMe Hot Plug Boot Optimized Storage Device</v>
       </c>
       <c r="D45" s="14">
         <v>1</v>
@@ -1666,13 +1666,13 @@
     </row>
     <row r="46">
       <c r="A46" s="8" t="str">
-        <v>P48832-B21</v>
+        <v>P52152-B21</v>
       </c>
       <c r="B46" s="9" t="str">
-        <v>Storage Cable</v>
+        <v>Boot Device</v>
       </c>
       <c r="C46" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 Tri-Mode Splitter Cable Kit</v>
+        <v>HPE ProLiant DL380 Gen11 NS204i-u Internal 40 Cable Kit</v>
       </c>
       <c r="D46" s="10">
         <v>1</v>
@@ -1686,13 +1686,13 @@
     </row>
     <row r="47">
       <c r="A47" s="12" t="str">
-        <v>P51911-B21</v>
+        <v>P54542-B21</v>
       </c>
       <c r="B47" s="13" t="str">
-        <v>OCP Enablement</v>
+        <v>Boot Device</v>
       </c>
       <c r="C47" s="13" t="str">
-        <v>HPE ProLiant DL360 Gen11 CPU1 to OCP2 x8 Enablement Kit</v>
+        <v>HPE ProLiant DL380 Gen11 NS204i-u FIO Bundle Kit</v>
       </c>
       <c r="D47" s="14">
         <v>1</v>
@@ -1706,13 +1706,13 @@
     </row>
     <row r="48">
       <c r="A48" s="8" t="str">
-        <v>P48830-B21</v>
+        <v>P48813-B21</v>
       </c>
       <c r="B48" s="9" t="str">
-        <v>OCP Enablement</v>
+        <v>Drive Cage</v>
       </c>
       <c r="C48" s="9" t="str">
-        <v>HPE ProLiant DL3XX Gen11 CPU2 to OCP2 x8 Enablement Kit</v>
+        <v>HPE ProLiant DL380 Gen11 2U 8SFF x1 Tri-Mode U.3 Drive Cage Kit</v>
       </c>
       <c r="D48" s="10">
         <v>1</v>
@@ -1726,13 +1726,13 @@
     </row>
     <row r="49">
       <c r="A49" s="12" t="str">
-        <v>P51181-B21</v>
+        <v>P48830-B21</v>
       </c>
       <c r="B49" s="13" t="str">
-        <v>Network Adapter</v>
+        <v>OCP Enablement</v>
       </c>
       <c r="C49" s="13" t="str">
-        <v>Broadcom BCM5719 Ethernet 1Gb 4-port BASE-T OCP3 Adapter for HPE</v>
+        <v>HPE ProLiant DL3XX Gen11 CPU2 to OCP2 x8 Enablement Kit</v>
       </c>
       <c r="D49" s="14">
         <v>1</v>
@@ -1746,13 +1746,13 @@
     </row>
     <row r="50">
       <c r="A50" s="8" t="str">
-        <v>P10115-B21</v>
+        <v>P51181-B21</v>
       </c>
       <c r="B50" s="9" t="str">
         <v>Network Adapter</v>
       </c>
       <c r="C50" s="9" t="str">
-        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 OCP3 Adapter for HPE</v>
+        <v>Broadcom BCM5719 Ethernet 1Gb 4-port BASE-T OCP3 Adapter for HPE</v>
       </c>
       <c r="D50" s="10">
         <v>1</v>
@@ -1766,93 +1766,93 @@
     </row>
     <row r="51">
       <c r="A51" s="12" t="str">
-        <v>P26262-B21</v>
+        <v>P10115-B21</v>
       </c>
       <c r="B51" s="13" t="str">
         <v>Network Adapter</v>
       </c>
       <c r="C51" s="13" t="str">
-        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 Adapter for HPE</v>
+        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 OCP3 Adapter for HPE</v>
       </c>
       <c r="D51" s="14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E51" s="16" t="str">
         <v/>
       </c>
       <c r="F51" s="14">
-        <v>120</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="8" t="str">
-        <v>845398-B21</v>
+        <v>P26262-B21</v>
       </c>
       <c r="B52" s="9" t="str">
-        <v>Transceiver</v>
+        <v>Network Adapter</v>
       </c>
       <c r="C52" s="9" t="str">
-        <v>HPE 25Gb SFP28 SR 100m Transceiver</v>
+        <v>Broadcom BCM57414 Ethernet 10/25Gb 2-port SFP28 Adapter for HPE</v>
       </c>
       <c r="D52" s="10">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E52" s="16" t="str">
         <v/>
       </c>
       <c r="F52" s="10">
-        <v>320</v>
+        <v>120</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="str">
-        <v>R2E09A</v>
+        <v>845398-B21</v>
       </c>
       <c r="B53" s="13" t="str">
-        <v>FC HBA</v>
+        <v>Transceiver</v>
       </c>
       <c r="C53" s="13" t="str">
-        <v>HPE SN1610Q 32Gb 2-port Fiber Channel Host Bus Adapter</v>
+        <v>HPE 25Gb SFP28 SR 100m Transceiver</v>
       </c>
       <c r="D53" s="14">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E53" s="16" t="str">
         <v/>
       </c>
       <c r="F53" s="14">
-        <v>80</v>
+        <v>320</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="str">
-        <v>P48803-B21</v>
+        <v>R2E09A</v>
       </c>
       <c r="B54" s="9" t="str">
-        <v>PCIe Riser</v>
+        <v>FC HBA</v>
       </c>
       <c r="C54" s="9" t="str">
-        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Primary Riser Kit</v>
+        <v>HPE SN1610Q 32Gb 2-port Fiber Channel Host Bus Adapter</v>
       </c>
       <c r="D54" s="10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E54" s="16" t="str">
         <v/>
       </c>
       <c r="F54" s="10">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="12" t="str">
-        <v>P51083-B21</v>
+        <v>P48803-B21</v>
       </c>
       <c r="B55" s="13" t="str">
         <v>PCIe Riser</v>
       </c>
       <c r="C55" s="13" t="str">
-        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Secondary Riser Kit</v>
+        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Primary Riser Kit</v>
       </c>
       <c r="D55" s="14">
         <v>1</v>
@@ -1866,13 +1866,13 @@
     </row>
     <row r="56">
       <c r="A56" s="8" t="str">
-        <v>P52341-B21</v>
+        <v>P56073-B21</v>
       </c>
       <c r="B56" s="9" t="str">
-        <v>Racking</v>
+        <v>PCIe Riser Cable</v>
       </c>
       <c r="C56" s="9" t="str">
-        <v>HPE ProLiant DL3XX Gen11 Easy Install Rail 3 Kit</v>
+        <v>HPE ProLiant DL380 Gen11 x16/x16/x16 Primary Cable Kit (Slot 1 Enablement)</v>
       </c>
       <c r="D56" s="10">
         <v>1</v>
@@ -1886,21 +1886,101 @@
     </row>
     <row r="57">
       <c r="A57" s="12" t="str">
+        <v>P51083-B21</v>
+      </c>
+      <c r="B57" s="13" t="str">
+        <v>PCIe Riser</v>
+      </c>
+      <c r="C57" s="13" t="str">
+        <v>HPE ProLiant DL380 Gen11 2U x16/x16/x16 Secondary Riser Kit</v>
+      </c>
+      <c r="D57" s="14">
+        <v>1</v>
+      </c>
+      <c r="E57" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F57" s="14">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="str">
+        <v>P56074-B21</v>
+      </c>
+      <c r="B58" s="9" t="str">
+        <v>PCIe Riser Cable</v>
+      </c>
+      <c r="C58" s="9" t="str">
+        <v>HPE ProLiant DL380 Gen11 x16/x16/x16 Secondary Cable Kit (Slot 4 Enablement)</v>
+      </c>
+      <c r="D58" s="10">
+        <v>1</v>
+      </c>
+      <c r="E58" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F58" s="10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="12" t="str">
+        <v>P52341-B21</v>
+      </c>
+      <c r="B59" s="13" t="str">
+        <v>Racking</v>
+      </c>
+      <c r="C59" s="13" t="str">
+        <v>HPE ProLiant DL3XX Gen11 Easy Install Rail 3 Kit</v>
+      </c>
+      <c r="D59" s="14">
+        <v>1</v>
+      </c>
+      <c r="E59" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F59" s="14">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="str">
         <v>P22020-B21</v>
       </c>
-      <c r="B57" s="13" t="str">
+      <c r="B60" s="9" t="str">
         <v>Racking</v>
       </c>
-      <c r="C57" s="13" t="str">
+      <c r="C60" s="9" t="str">
         <v>HPE DL38X Gen10 Plus 2U Cable Management Arm for Rail Kit</v>
       </c>
-      <c r="D57" s="14">
-        <v>1</v>
-      </c>
-      <c r="E57" s="16" t="str">
-        <v/>
-      </c>
-      <c r="F57" s="14">
+      <c r="D60" s="10">
+        <v>1</v>
+      </c>
+      <c r="E60" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F60" s="10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="12" t="str">
+        <v>R7A11AAE</v>
+      </c>
+      <c r="B61" s="13" t="str">
+        <v>Management License</v>
+      </c>
+      <c r="C61" s="13" t="str">
+        <v>HPE Compute Ops Management Enhanced 3-year SaaS</v>
+      </c>
+      <c r="D61" s="14">
+        <v>1</v>
+      </c>
+      <c r="E61" s="16" t="str">
+        <v/>
+      </c>
+      <c r="F61" s="14">
         <v>40</v>
       </c>
     </row>
@@ -1909,12 +1989,12 @@
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="E6:E29"/>
-    <mergeCell ref="A32:F32"/>
-    <mergeCell ref="E34:E57"/>
+    <mergeCell ref="E6:E31"/>
+    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="E36:E61"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F57"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>